<commit_message>
Actualizar plantilla F-MAN-008 (nueva version con campo Consecutivo) y escribir el consecutivo en su celda
</commit_message>
<xml_diff>
--- a/assets/fman008_template.xlsx
+++ b/assets/fman008_template.xlsx
@@ -5,7 +5,7 @@
   <workbookPr defaultThemeVersion="153222"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\172.20.48.16\sistemas de calidad interna\0.0 PLANTA PLATINO\MANTENIMIENTO\FORMATOS\EN TRÁMITE\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\victor.veru\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="65" uniqueCount="58">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="66" uniqueCount="59">
   <si>
     <t>NOMBRE DE LA EMPRESA:</t>
   </si>
@@ -241,6 +241,9 @@
   </si>
   <si>
     <t>CÓDIGO: F-MAN-008                VERSIÓN: 02              FECHA DE APLICACIÓN:  01-08-2024</t>
+  </si>
+  <si>
+    <t>CONSECUTIVO</t>
   </si>
 </sst>
 </file>
@@ -1131,6 +1134,15 @@
     <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="39" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
@@ -1305,18 +1317,6 @@
     <xf numFmtId="0" fontId="10" fillId="0" borderId="27" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="12" fillId="0" borderId="32" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -1403,6 +1403,9 @@
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="28" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1729,107 +1732,109 @@
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:N97"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="11.453125" defaultRowHeight="14" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="11.42578125" style="2"/>
+    <col min="1" max="1" width="11.453125" style="2"/>
     <col min="2" max="2" width="16" style="2" customWidth="1"/>
-    <col min="3" max="3" width="15.28515625" style="2" customWidth="1"/>
-    <col min="4" max="4" width="11.7109375" style="2" customWidth="1"/>
-    <col min="5" max="5" width="13.42578125" style="2" customWidth="1"/>
-    <col min="6" max="6" width="11.7109375" style="2" customWidth="1"/>
-    <col min="7" max="7" width="18.7109375" style="2" customWidth="1"/>
-    <col min="8" max="8" width="5.7109375" style="2" customWidth="1"/>
-    <col min="9" max="9" width="9.140625" style="2" customWidth="1"/>
-    <col min="10" max="10" width="10.42578125" style="2" customWidth="1"/>
-    <col min="11" max="11" width="3.42578125" style="2" customWidth="1"/>
-    <col min="12" max="12" width="7.85546875" style="2" customWidth="1"/>
-    <col min="13" max="13" width="12.5703125" style="2" customWidth="1"/>
-    <col min="14" max="14" width="5.7109375" style="2" customWidth="1"/>
-    <col min="15" max="16384" width="11.42578125" style="2"/>
+    <col min="3" max="3" width="15.26953125" style="2" customWidth="1"/>
+    <col min="4" max="4" width="11.7265625" style="2" customWidth="1"/>
+    <col min="5" max="5" width="13.453125" style="2" customWidth="1"/>
+    <col min="6" max="6" width="11.7265625" style="2" customWidth="1"/>
+    <col min="7" max="7" width="18.7265625" style="2" customWidth="1"/>
+    <col min="8" max="8" width="5.7265625" style="2" customWidth="1"/>
+    <col min="9" max="9" width="9.1796875" style="2" customWidth="1"/>
+    <col min="10" max="10" width="14.90625" style="2" customWidth="1"/>
+    <col min="11" max="11" width="3.453125" style="2" customWidth="1"/>
+    <col min="12" max="12" width="7.81640625" style="2" customWidth="1"/>
+    <col min="13" max="13" width="12.54296875" style="2" customWidth="1"/>
+    <col min="14" max="14" width="5.7265625" style="2" customWidth="1"/>
+    <col min="15" max="16384" width="11.453125" style="2"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:13" ht="20.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="107" t="s">
+    <row r="1" spans="1:13" ht="20.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A1" s="49" t="s">
         <v>30</v>
       </c>
-      <c r="B1" s="108"/>
-      <c r="C1" s="108"/>
-      <c r="D1" s="108"/>
-      <c r="E1" s="108"/>
-      <c r="F1" s="108"/>
-      <c r="G1" s="108"/>
-      <c r="H1" s="108"/>
-      <c r="I1" s="109"/>
-      <c r="J1" s="109"/>
-      <c r="K1" s="109"/>
-      <c r="L1" s="110"/>
-      <c r="M1" s="111"/>
-    </row>
-    <row r="2" spans="1:13" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="114" t="s">
+      <c r="B1" s="50"/>
+      <c r="C1" s="50"/>
+      <c r="D1" s="50"/>
+      <c r="E1" s="50"/>
+      <c r="F1" s="50"/>
+      <c r="G1" s="50"/>
+      <c r="H1" s="50"/>
+      <c r="I1" s="50"/>
+      <c r="J1" s="139" t="s">
+        <v>58</v>
+      </c>
+      <c r="K1" s="49"/>
+      <c r="L1" s="51"/>
+      <c r="M1" s="110"/>
+    </row>
+    <row r="2" spans="1:13" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A2" s="113" t="s">
         <v>0</v>
       </c>
-      <c r="B2" s="115"/>
-      <c r="C2" s="116"/>
-      <c r="D2" s="123" t="s">
+      <c r="B2" s="114"/>
+      <c r="C2" s="115"/>
+      <c r="D2" s="122" t="s">
         <v>21</v>
       </c>
-      <c r="E2" s="124"/>
-      <c r="F2" s="124"/>
-      <c r="G2" s="124"/>
-      <c r="H2" s="124"/>
-      <c r="I2" s="125" t="s">
+      <c r="E2" s="123"/>
+      <c r="F2" s="123"/>
+      <c r="G2" s="123"/>
+      <c r="H2" s="123"/>
+      <c r="I2" s="124" t="s">
         <v>6</v>
       </c>
-      <c r="J2" s="126"/>
-      <c r="K2" s="126"/>
-      <c r="L2" s="127"/>
-      <c r="M2" s="112"/>
-    </row>
-    <row r="3" spans="1:13" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="117" t="s">
+      <c r="J2" s="125"/>
+      <c r="K2" s="125"/>
+      <c r="L2" s="126"/>
+      <c r="M2" s="111"/>
+    </row>
+    <row r="3" spans="1:13" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A3" s="116" t="s">
         <v>56</v>
       </c>
-      <c r="B3" s="118"/>
-      <c r="C3" s="119"/>
-      <c r="D3" s="134" t="s">
+      <c r="B3" s="117"/>
+      <c r="C3" s="118"/>
+      <c r="D3" s="133" t="s">
         <v>22</v>
       </c>
-      <c r="E3" s="135"/>
-      <c r="F3" s="135"/>
-      <c r="G3" s="136"/>
+      <c r="E3" s="134"/>
+      <c r="F3" s="134"/>
+      <c r="G3" s="135"/>
       <c r="H3" s="20"/>
-      <c r="I3" s="128"/>
-      <c r="J3" s="129"/>
-      <c r="K3" s="129"/>
-      <c r="L3" s="130"/>
-      <c r="M3" s="112"/>
-    </row>
-    <row r="4" spans="1:13" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="120"/>
-      <c r="B4" s="121"/>
-      <c r="C4" s="122"/>
-      <c r="D4" s="137" t="s">
+      <c r="I3" s="127"/>
+      <c r="J3" s="128"/>
+      <c r="K3" s="128"/>
+      <c r="L3" s="129"/>
+      <c r="M3" s="111"/>
+    </row>
+    <row r="4" spans="1:13" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A4" s="119"/>
+      <c r="B4" s="120"/>
+      <c r="C4" s="121"/>
+      <c r="D4" s="136" t="s">
         <v>23</v>
       </c>
-      <c r="E4" s="138"/>
-      <c r="F4" s="138"/>
-      <c r="G4" s="139"/>
+      <c r="E4" s="137"/>
+      <c r="F4" s="137"/>
+      <c r="G4" s="138"/>
       <c r="H4" s="18"/>
       <c r="I4" s="19" t="s">
         <v>16</v>
       </c>
-      <c r="J4" s="131"/>
-      <c r="K4" s="132"/>
-      <c r="L4" s="133"/>
-      <c r="M4" s="113"/>
-    </row>
-    <row r="5" spans="1:13" ht="25.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="J4" s="130"/>
+      <c r="K4" s="131"/>
+      <c r="L4" s="132"/>
+      <c r="M4" s="112"/>
+    </row>
+    <row r="5" spans="1:13" ht="25.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A5" s="15" t="s">
         <v>12</v>
       </c>
-      <c r="B5" s="72"/>
-      <c r="C5" s="73"/>
+      <c r="B5" s="75"/>
+      <c r="C5" s="76"/>
       <c r="D5" s="16" t="s">
         <v>17</v>
       </c>
@@ -1838,118 +1843,118 @@
         <v>1</v>
       </c>
       <c r="G5" s="30"/>
-      <c r="H5" s="74" t="s">
+      <c r="H5" s="77" t="s">
         <v>18</v>
       </c>
-      <c r="I5" s="75"/>
+      <c r="I5" s="78"/>
       <c r="J5" s="31" t="s">
         <v>20</v>
       </c>
-      <c r="K5" s="76" t="s">
+      <c r="K5" s="79" t="s">
         <v>15</v>
       </c>
-      <c r="L5" s="77"/>
+      <c r="L5" s="80"/>
       <c r="M5" s="32"/>
     </row>
-    <row r="6" spans="1:13" ht="18" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A6" s="101" t="s">
+    <row r="6" spans="1:13" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A6" s="104" t="s">
         <v>34</v>
       </c>
-      <c r="B6" s="102"/>
-      <c r="C6" s="102"/>
-      <c r="D6" s="102"/>
-      <c r="E6" s="102"/>
-      <c r="F6" s="102"/>
-      <c r="G6" s="102"/>
-      <c r="H6" s="102"/>
-      <c r="I6" s="102"/>
-      <c r="J6" s="99"/>
-      <c r="K6" s="102"/>
-      <c r="L6" s="102"/>
-      <c r="M6" s="103"/>
-    </row>
-    <row r="7" spans="1:13" ht="28.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A7" s="104"/>
-      <c r="B7" s="105"/>
-      <c r="C7" s="105"/>
-      <c r="D7" s="105"/>
-      <c r="E7" s="105"/>
-      <c r="F7" s="105"/>
-      <c r="G7" s="105"/>
-      <c r="H7" s="105"/>
-      <c r="I7" s="105"/>
-      <c r="J7" s="105"/>
-      <c r="K7" s="105"/>
-      <c r="L7" s="105"/>
-      <c r="M7" s="106"/>
-    </row>
-    <row r="8" spans="1:13" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A8" s="95" t="s">
+      <c r="B6" s="105"/>
+      <c r="C6" s="105"/>
+      <c r="D6" s="105"/>
+      <c r="E6" s="105"/>
+      <c r="F6" s="105"/>
+      <c r="G6" s="105"/>
+      <c r="H6" s="105"/>
+      <c r="I6" s="105"/>
+      <c r="J6" s="102"/>
+      <c r="K6" s="105"/>
+      <c r="L6" s="105"/>
+      <c r="M6" s="106"/>
+    </row>
+    <row r="7" spans="1:13" ht="28.5" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A7" s="107"/>
+      <c r="B7" s="108"/>
+      <c r="C7" s="108"/>
+      <c r="D7" s="108"/>
+      <c r="E7" s="108"/>
+      <c r="F7" s="108"/>
+      <c r="G7" s="108"/>
+      <c r="H7" s="108"/>
+      <c r="I7" s="108"/>
+      <c r="J7" s="108"/>
+      <c r="K7" s="108"/>
+      <c r="L7" s="108"/>
+      <c r="M7" s="109"/>
+    </row>
+    <row r="8" spans="1:13" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A8" s="98" t="s">
         <v>35</v>
       </c>
-      <c r="B8" s="96"/>
-      <c r="C8" s="96"/>
-      <c r="D8" s="96"/>
-      <c r="E8" s="96"/>
-      <c r="F8" s="96"/>
-      <c r="G8" s="96"/>
-      <c r="H8" s="96"/>
-      <c r="I8" s="96"/>
-      <c r="J8" s="96"/>
-      <c r="K8" s="96"/>
-      <c r="L8" s="96"/>
-      <c r="M8" s="97"/>
-    </row>
-    <row r="9" spans="1:13" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A9" s="98"/>
-      <c r="B9" s="99"/>
-      <c r="C9" s="99"/>
-      <c r="D9" s="99"/>
-      <c r="E9" s="99"/>
-      <c r="F9" s="99"/>
-      <c r="G9" s="99"/>
-      <c r="H9" s="99"/>
-      <c r="I9" s="99"/>
-      <c r="J9" s="99"/>
-      <c r="K9" s="99"/>
-      <c r="L9" s="99"/>
-      <c r="M9" s="100"/>
-    </row>
-    <row r="10" spans="1:13" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A10" s="69" t="s">
+      <c r="B8" s="99"/>
+      <c r="C8" s="99"/>
+      <c r="D8" s="99"/>
+      <c r="E8" s="99"/>
+      <c r="F8" s="99"/>
+      <c r="G8" s="99"/>
+      <c r="H8" s="99"/>
+      <c r="I8" s="99"/>
+      <c r="J8" s="99"/>
+      <c r="K8" s="99"/>
+      <c r="L8" s="99"/>
+      <c r="M8" s="100"/>
+    </row>
+    <row r="9" spans="1:13" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A9" s="101"/>
+      <c r="B9" s="102"/>
+      <c r="C9" s="102"/>
+      <c r="D9" s="102"/>
+      <c r="E9" s="102"/>
+      <c r="F9" s="102"/>
+      <c r="G9" s="102"/>
+      <c r="H9" s="102"/>
+      <c r="I9" s="102"/>
+      <c r="J9" s="102"/>
+      <c r="K9" s="102"/>
+      <c r="L9" s="102"/>
+      <c r="M9" s="103"/>
+    </row>
+    <row r="10" spans="1:13" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A10" s="72" t="s">
         <v>19</v>
       </c>
-      <c r="B10" s="80" t="s">
+      <c r="B10" s="83" t="s">
         <v>2</v>
       </c>
-      <c r="C10" s="80"/>
-      <c r="D10" s="80"/>
-      <c r="E10" s="80"/>
-      <c r="F10" s="80"/>
-      <c r="G10" s="80"/>
-      <c r="H10" s="80"/>
-      <c r="I10" s="80"/>
-      <c r="J10" s="80"/>
-      <c r="K10" s="81"/>
-      <c r="L10" s="78" t="s">
+      <c r="C10" s="83"/>
+      <c r="D10" s="83"/>
+      <c r="E10" s="83"/>
+      <c r="F10" s="83"/>
+      <c r="G10" s="83"/>
+      <c r="H10" s="83"/>
+      <c r="I10" s="83"/>
+      <c r="J10" s="83"/>
+      <c r="K10" s="84"/>
+      <c r="L10" s="81" t="s">
         <v>3</v>
       </c>
-      <c r="M10" s="79"/>
-    </row>
-    <row r="11" spans="1:13" ht="15" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A11" s="70"/>
-      <c r="B11" s="82" t="s">
+      <c r="M10" s="82"/>
+    </row>
+    <row r="11" spans="1:13" ht="14.5" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A11" s="73"/>
+      <c r="B11" s="85" t="s">
         <v>24</v>
       </c>
-      <c r="C11" s="83"/>
-      <c r="D11" s="83"/>
-      <c r="E11" s="83"/>
-      <c r="F11" s="83"/>
-      <c r="G11" s="83"/>
-      <c r="H11" s="83"/>
-      <c r="I11" s="83"/>
-      <c r="J11" s="83"/>
-      <c r="K11" s="84"/>
+      <c r="C11" s="86"/>
+      <c r="D11" s="86"/>
+      <c r="E11" s="86"/>
+      <c r="F11" s="86"/>
+      <c r="G11" s="86"/>
+      <c r="H11" s="86"/>
+      <c r="I11" s="86"/>
+      <c r="J11" s="86"/>
+      <c r="K11" s="87"/>
       <c r="L11" s="13" t="s">
         <v>7</v>
       </c>
@@ -1957,156 +1962,156 @@
         <v>8</v>
       </c>
     </row>
-    <row r="12" spans="1:13" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A12" s="70"/>
-      <c r="B12" s="64" t="s">
+    <row r="12" spans="1:13" ht="22.5" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A12" s="73"/>
+      <c r="B12" s="67" t="s">
         <v>36</v>
       </c>
-      <c r="C12" s="65"/>
-      <c r="D12" s="65"/>
-      <c r="E12" s="65"/>
-      <c r="F12" s="65"/>
-      <c r="G12" s="65"/>
-      <c r="H12" s="65"/>
-      <c r="I12" s="65"/>
-      <c r="J12" s="65"/>
+      <c r="C12" s="68"/>
+      <c r="D12" s="68"/>
+      <c r="E12" s="68"/>
+      <c r="F12" s="68"/>
+      <c r="G12" s="68"/>
+      <c r="H12" s="68"/>
+      <c r="I12" s="68"/>
+      <c r="J12" s="68"/>
       <c r="K12" s="26"/>
       <c r="L12" s="28"/>
       <c r="M12" s="33"/>
     </row>
-    <row r="13" spans="1:13" ht="26.1" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A13" s="70"/>
-      <c r="B13" s="49" t="s">
+    <row r="13" spans="1:13" ht="26.15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A13" s="73"/>
+      <c r="B13" s="52" t="s">
         <v>37</v>
       </c>
-      <c r="C13" s="50"/>
-      <c r="D13" s="50"/>
-      <c r="E13" s="50"/>
-      <c r="F13" s="50"/>
-      <c r="G13" s="50"/>
-      <c r="H13" s="50"/>
-      <c r="I13" s="50"/>
-      <c r="J13" s="50"/>
+      <c r="C13" s="53"/>
+      <c r="D13" s="53"/>
+      <c r="E13" s="53"/>
+      <c r="F13" s="53"/>
+      <c r="G13" s="53"/>
+      <c r="H13" s="53"/>
+      <c r="I13" s="53"/>
+      <c r="J13" s="53"/>
       <c r="K13" s="25"/>
       <c r="L13" s="28"/>
       <c r="M13" s="33"/>
     </row>
-    <row r="14" spans="1:13" ht="23.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A14" s="70"/>
-      <c r="B14" s="49" t="s">
+    <row r="14" spans="1:13" ht="23.25" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A14" s="73"/>
+      <c r="B14" s="52" t="s">
         <v>38</v>
       </c>
-      <c r="C14" s="50"/>
-      <c r="D14" s="50"/>
-      <c r="E14" s="50"/>
-      <c r="F14" s="50"/>
-      <c r="G14" s="50"/>
-      <c r="H14" s="50"/>
-      <c r="I14" s="50"/>
-      <c r="J14" s="50"/>
+      <c r="C14" s="53"/>
+      <c r="D14" s="53"/>
+      <c r="E14" s="53"/>
+      <c r="F14" s="53"/>
+      <c r="G14" s="53"/>
+      <c r="H14" s="53"/>
+      <c r="I14" s="53"/>
+      <c r="J14" s="53"/>
       <c r="K14" s="36"/>
       <c r="L14" s="9"/>
       <c r="M14" s="10"/>
     </row>
-    <row r="15" spans="1:13" ht="15.95" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A15" s="70"/>
-      <c r="B15" s="49" t="s">
+    <row r="15" spans="1:13" ht="16" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A15" s="73"/>
+      <c r="B15" s="52" t="s">
         <v>39</v>
       </c>
-      <c r="C15" s="50"/>
-      <c r="D15" s="50"/>
-      <c r="E15" s="50"/>
-      <c r="F15" s="50"/>
-      <c r="G15" s="50"/>
-      <c r="H15" s="50"/>
-      <c r="I15" s="50"/>
-      <c r="J15" s="50"/>
+      <c r="C15" s="53"/>
+      <c r="D15" s="53"/>
+      <c r="E15" s="53"/>
+      <c r="F15" s="53"/>
+      <c r="G15" s="53"/>
+      <c r="H15" s="53"/>
+      <c r="I15" s="53"/>
+      <c r="J15" s="53"/>
       <c r="K15" s="25"/>
       <c r="L15" s="28"/>
       <c r="M15" s="33"/>
     </row>
-    <row r="16" spans="1:13" ht="15.95" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A16" s="70"/>
-      <c r="B16" s="49" t="s">
+    <row r="16" spans="1:13" ht="16" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A16" s="73"/>
+      <c r="B16" s="52" t="s">
         <v>40</v>
       </c>
-      <c r="C16" s="50"/>
-      <c r="D16" s="50"/>
-      <c r="E16" s="50"/>
-      <c r="F16" s="50"/>
-      <c r="G16" s="50"/>
-      <c r="H16" s="50"/>
-      <c r="I16" s="50"/>
-      <c r="J16" s="50"/>
+      <c r="C16" s="53"/>
+      <c r="D16" s="53"/>
+      <c r="E16" s="53"/>
+      <c r="F16" s="53"/>
+      <c r="G16" s="53"/>
+      <c r="H16" s="53"/>
+      <c r="I16" s="53"/>
+      <c r="J16" s="53"/>
       <c r="K16" s="25"/>
       <c r="L16" s="28"/>
       <c r="M16" s="33"/>
     </row>
-    <row r="17" spans="1:13" ht="21.95" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A17" s="70"/>
-      <c r="B17" s="49" t="s">
+    <row r="17" spans="1:13" ht="22" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A17" s="73"/>
+      <c r="B17" s="52" t="s">
         <v>41</v>
       </c>
-      <c r="C17" s="50"/>
-      <c r="D17" s="50"/>
-      <c r="E17" s="50"/>
-      <c r="F17" s="50"/>
-      <c r="G17" s="50"/>
-      <c r="H17" s="50"/>
-      <c r="I17" s="50"/>
-      <c r="J17" s="50"/>
+      <c r="C17" s="53"/>
+      <c r="D17" s="53"/>
+      <c r="E17" s="53"/>
+      <c r="F17" s="53"/>
+      <c r="G17" s="53"/>
+      <c r="H17" s="53"/>
+      <c r="I17" s="53"/>
+      <c r="J17" s="53"/>
       <c r="K17" s="25"/>
       <c r="L17" s="28"/>
       <c r="M17" s="33"/>
     </row>
-    <row r="18" spans="1:13" ht="15.95" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A18" s="70"/>
-      <c r="B18" s="49" t="s">
+    <row r="18" spans="1:13" ht="16" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A18" s="73"/>
+      <c r="B18" s="52" t="s">
         <v>42</v>
       </c>
-      <c r="C18" s="50"/>
-      <c r="D18" s="50"/>
-      <c r="E18" s="50"/>
-      <c r="F18" s="50"/>
-      <c r="G18" s="50"/>
-      <c r="H18" s="50"/>
-      <c r="I18" s="50"/>
-      <c r="J18" s="50"/>
+      <c r="C18" s="53"/>
+      <c r="D18" s="53"/>
+      <c r="E18" s="53"/>
+      <c r="F18" s="53"/>
+      <c r="G18" s="53"/>
+      <c r="H18" s="53"/>
+      <c r="I18" s="53"/>
+      <c r="J18" s="53"/>
       <c r="K18" s="25"/>
       <c r="L18" s="28"/>
       <c r="M18" s="33"/>
     </row>
-    <row r="19" spans="1:13" ht="18.95" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A19" s="70"/>
-      <c r="B19" s="62" t="s">
+    <row r="19" spans="1:13" ht="19" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A19" s="73"/>
+      <c r="B19" s="65" t="s">
         <v>43</v>
       </c>
-      <c r="C19" s="63"/>
-      <c r="D19" s="63"/>
-      <c r="E19" s="63"/>
-      <c r="F19" s="63"/>
-      <c r="G19" s="63"/>
-      <c r="H19" s="63"/>
-      <c r="I19" s="63"/>
-      <c r="J19" s="63"/>
+      <c r="C19" s="66"/>
+      <c r="D19" s="66"/>
+      <c r="E19" s="66"/>
+      <c r="F19" s="66"/>
+      <c r="G19" s="66"/>
+      <c r="H19" s="66"/>
+      <c r="I19" s="66"/>
+      <c r="J19" s="66"/>
       <c r="K19" s="27"/>
       <c r="L19" s="28"/>
       <c r="M19" s="33"/>
     </row>
-    <row r="20" spans="1:13" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A20" s="70"/>
-      <c r="B20" s="85" t="s">
+    <row r="20" spans="1:13" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A20" s="73"/>
+      <c r="B20" s="88" t="s">
         <v>25</v>
       </c>
-      <c r="C20" s="86"/>
-      <c r="D20" s="86"/>
-      <c r="E20" s="86"/>
-      <c r="F20" s="86"/>
-      <c r="G20" s="86"/>
-      <c r="H20" s="86"/>
-      <c r="I20" s="86"/>
-      <c r="J20" s="86"/>
-      <c r="K20" s="87"/>
+      <c r="C20" s="89"/>
+      <c r="D20" s="89"/>
+      <c r="E20" s="89"/>
+      <c r="F20" s="89"/>
+      <c r="G20" s="89"/>
+      <c r="H20" s="89"/>
+      <c r="I20" s="89"/>
+      <c r="J20" s="89"/>
+      <c r="K20" s="90"/>
       <c r="L20" s="14" t="s">
         <v>7</v>
       </c>
@@ -2114,224 +2119,224 @@
         <v>8</v>
       </c>
     </row>
-    <row r="21" spans="1:13" ht="34.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A21" s="70"/>
-      <c r="B21" s="64" t="s">
+    <row r="21" spans="1:13" ht="34.5" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A21" s="73"/>
+      <c r="B21" s="67" t="s">
         <v>44</v>
       </c>
-      <c r="C21" s="65"/>
-      <c r="D21" s="65"/>
-      <c r="E21" s="65"/>
-      <c r="F21" s="65"/>
-      <c r="G21" s="65"/>
-      <c r="H21" s="65"/>
-      <c r="I21" s="65"/>
-      <c r="J21" s="65"/>
+      <c r="C21" s="68"/>
+      <c r="D21" s="68"/>
+      <c r="E21" s="68"/>
+      <c r="F21" s="68"/>
+      <c r="G21" s="68"/>
+      <c r="H21" s="68"/>
+      <c r="I21" s="68"/>
+      <c r="J21" s="68"/>
       <c r="K21" s="26"/>
       <c r="L21" s="28"/>
       <c r="M21" s="33"/>
     </row>
-    <row r="22" spans="1:13" ht="14.1" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A22" s="70"/>
-      <c r="B22" s="49" t="s">
+    <row r="22" spans="1:13" ht="14.15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A22" s="73"/>
+      <c r="B22" s="52" t="s">
         <v>13</v>
       </c>
-      <c r="C22" s="50"/>
-      <c r="D22" s="50"/>
-      <c r="E22" s="50"/>
-      <c r="F22" s="50"/>
-      <c r="G22" s="50"/>
-      <c r="H22" s="50"/>
-      <c r="I22" s="50"/>
-      <c r="J22" s="50"/>
+      <c r="C22" s="53"/>
+      <c r="D22" s="53"/>
+      <c r="E22" s="53"/>
+      <c r="F22" s="53"/>
+      <c r="G22" s="53"/>
+      <c r="H22" s="53"/>
+      <c r="I22" s="53"/>
+      <c r="J22" s="53"/>
       <c r="K22" s="25"/>
       <c r="L22" s="28"/>
       <c r="M22" s="33"/>
     </row>
-    <row r="23" spans="1:13" ht="21" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A23" s="70"/>
-      <c r="B23" s="49" t="s">
+    <row r="23" spans="1:13" ht="21" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A23" s="73"/>
+      <c r="B23" s="52" t="s">
         <v>45</v>
       </c>
-      <c r="C23" s="50"/>
-      <c r="D23" s="50"/>
-      <c r="E23" s="50"/>
-      <c r="F23" s="50"/>
-      <c r="G23" s="50"/>
-      <c r="H23" s="50"/>
-      <c r="I23" s="50"/>
-      <c r="J23" s="50"/>
+      <c r="C23" s="53"/>
+      <c r="D23" s="53"/>
+      <c r="E23" s="53"/>
+      <c r="F23" s="53"/>
+      <c r="G23" s="53"/>
+      <c r="H23" s="53"/>
+      <c r="I23" s="53"/>
+      <c r="J23" s="53"/>
       <c r="K23" s="25"/>
       <c r="L23" s="28"/>
       <c r="M23" s="33"/>
     </row>
-    <row r="24" spans="1:13" ht="21.95" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A24" s="70"/>
-      <c r="B24" s="49" t="s">
+    <row r="24" spans="1:13" ht="22" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A24" s="73"/>
+      <c r="B24" s="52" t="s">
         <v>46</v>
       </c>
-      <c r="C24" s="50"/>
-      <c r="D24" s="50"/>
-      <c r="E24" s="50"/>
-      <c r="F24" s="50"/>
-      <c r="G24" s="50"/>
-      <c r="H24" s="50"/>
-      <c r="I24" s="50"/>
-      <c r="J24" s="50"/>
+      <c r="C24" s="53"/>
+      <c r="D24" s="53"/>
+      <c r="E24" s="53"/>
+      <c r="F24" s="53"/>
+      <c r="G24" s="53"/>
+      <c r="H24" s="53"/>
+      <c r="I24" s="53"/>
+      <c r="J24" s="53"/>
       <c r="K24" s="25"/>
       <c r="L24" s="28"/>
       <c r="M24" s="33"/>
     </row>
-    <row r="25" spans="1:13" ht="14.1" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A25" s="70"/>
-      <c r="B25" s="49" t="s">
+    <row r="25" spans="1:13" ht="14.15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A25" s="73"/>
+      <c r="B25" s="52" t="s">
         <v>47</v>
       </c>
-      <c r="C25" s="50"/>
-      <c r="D25" s="50"/>
-      <c r="E25" s="50"/>
-      <c r="F25" s="50"/>
-      <c r="G25" s="50"/>
-      <c r="H25" s="50"/>
-      <c r="I25" s="50"/>
-      <c r="J25" s="50"/>
+      <c r="C25" s="53"/>
+      <c r="D25" s="53"/>
+      <c r="E25" s="53"/>
+      <c r="F25" s="53"/>
+      <c r="G25" s="53"/>
+      <c r="H25" s="53"/>
+      <c r="I25" s="53"/>
+      <c r="J25" s="53"/>
       <c r="K25" s="25"/>
       <c r="L25" s="28"/>
       <c r="M25" s="33"/>
     </row>
-    <row r="26" spans="1:13" ht="14.1" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A26" s="70"/>
-      <c r="B26" s="49" t="s">
+    <row r="26" spans="1:13" ht="14.15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A26" s="73"/>
+      <c r="B26" s="52" t="s">
         <v>28</v>
       </c>
-      <c r="C26" s="50"/>
-      <c r="D26" s="50"/>
-      <c r="E26" s="50"/>
-      <c r="F26" s="50"/>
-      <c r="G26" s="50"/>
-      <c r="H26" s="50"/>
-      <c r="I26" s="50"/>
-      <c r="J26" s="50"/>
+      <c r="C26" s="53"/>
+      <c r="D26" s="53"/>
+      <c r="E26" s="53"/>
+      <c r="F26" s="53"/>
+      <c r="G26" s="53"/>
+      <c r="H26" s="53"/>
+      <c r="I26" s="53"/>
+      <c r="J26" s="53"/>
       <c r="K26" s="25"/>
       <c r="L26" s="28"/>
       <c r="M26" s="33"/>
     </row>
-    <row r="27" spans="1:13" ht="14.1" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A27" s="70"/>
-      <c r="B27" s="49" t="s">
+    <row r="27" spans="1:13" ht="14.15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A27" s="73"/>
+      <c r="B27" s="52" t="s">
         <v>48</v>
       </c>
-      <c r="C27" s="50"/>
-      <c r="D27" s="50"/>
-      <c r="E27" s="50"/>
-      <c r="F27" s="50"/>
-      <c r="G27" s="50"/>
-      <c r="H27" s="50"/>
-      <c r="I27" s="50"/>
-      <c r="J27" s="50"/>
+      <c r="C27" s="53"/>
+      <c r="D27" s="53"/>
+      <c r="E27" s="53"/>
+      <c r="F27" s="53"/>
+      <c r="G27" s="53"/>
+      <c r="H27" s="53"/>
+      <c r="I27" s="53"/>
+      <c r="J27" s="53"/>
       <c r="K27" s="25"/>
       <c r="L27" s="28"/>
       <c r="M27" s="33"/>
     </row>
-    <row r="28" spans="1:13" ht="14.1" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A28" s="70"/>
-      <c r="B28" s="49" t="s">
+    <row r="28" spans="1:13" ht="14.15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A28" s="73"/>
+      <c r="B28" s="52" t="s">
         <v>49</v>
       </c>
-      <c r="C28" s="50"/>
-      <c r="D28" s="50"/>
-      <c r="E28" s="50"/>
-      <c r="F28" s="50"/>
-      <c r="G28" s="50"/>
-      <c r="H28" s="50"/>
-      <c r="I28" s="50"/>
-      <c r="J28" s="50"/>
+      <c r="C28" s="53"/>
+      <c r="D28" s="53"/>
+      <c r="E28" s="53"/>
+      <c r="F28" s="53"/>
+      <c r="G28" s="53"/>
+      <c r="H28" s="53"/>
+      <c r="I28" s="53"/>
+      <c r="J28" s="53"/>
       <c r="K28" s="36"/>
       <c r="L28" s="28"/>
       <c r="M28" s="33"/>
     </row>
-    <row r="29" spans="1:13" ht="14.1" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A29" s="70"/>
-      <c r="B29" s="49" t="s">
+    <row r="29" spans="1:13" ht="14.15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A29" s="73"/>
+      <c r="B29" s="52" t="s">
         <v>50</v>
       </c>
-      <c r="C29" s="50"/>
-      <c r="D29" s="50"/>
-      <c r="E29" s="50"/>
-      <c r="F29" s="50"/>
-      <c r="G29" s="50"/>
-      <c r="H29" s="50"/>
-      <c r="I29" s="50"/>
-      <c r="J29" s="50"/>
+      <c r="C29" s="53"/>
+      <c r="D29" s="53"/>
+      <c r="E29" s="53"/>
+      <c r="F29" s="53"/>
+      <c r="G29" s="53"/>
+      <c r="H29" s="53"/>
+      <c r="I29" s="53"/>
+      <c r="J29" s="53"/>
       <c r="K29" s="25"/>
       <c r="L29" s="28"/>
       <c r="M29" s="33"/>
     </row>
-    <row r="30" spans="1:13" ht="23.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A30" s="70"/>
-      <c r="B30" s="49" t="s">
+    <row r="30" spans="1:13" ht="23.25" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A30" s="73"/>
+      <c r="B30" s="52" t="s">
         <v>51</v>
       </c>
-      <c r="C30" s="50"/>
-      <c r="D30" s="50"/>
-      <c r="E30" s="50"/>
-      <c r="F30" s="50"/>
-      <c r="G30" s="50"/>
-      <c r="H30" s="50"/>
-      <c r="I30" s="50"/>
-      <c r="J30" s="50"/>
+      <c r="C30" s="53"/>
+      <c r="D30" s="53"/>
+      <c r="E30" s="53"/>
+      <c r="F30" s="53"/>
+      <c r="G30" s="53"/>
+      <c r="H30" s="53"/>
+      <c r="I30" s="53"/>
+      <c r="J30" s="53"/>
       <c r="K30" s="25"/>
       <c r="L30" s="28"/>
       <c r="M30" s="33"/>
     </row>
-    <row r="31" spans="1:13" ht="19.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A31" s="70"/>
-      <c r="B31" s="49" t="s">
+    <row r="31" spans="1:13" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A31" s="73"/>
+      <c r="B31" s="52" t="s">
         <v>52</v>
       </c>
-      <c r="C31" s="50"/>
-      <c r="D31" s="50"/>
-      <c r="E31" s="50"/>
-      <c r="F31" s="50"/>
-      <c r="G31" s="50"/>
-      <c r="H31" s="50"/>
-      <c r="I31" s="50"/>
-      <c r="J31" s="50"/>
+      <c r="C31" s="53"/>
+      <c r="D31" s="53"/>
+      <c r="E31" s="53"/>
+      <c r="F31" s="53"/>
+      <c r="G31" s="53"/>
+      <c r="H31" s="53"/>
+      <c r="I31" s="53"/>
+      <c r="J31" s="53"/>
       <c r="K31" s="25"/>
       <c r="L31" s="28"/>
       <c r="M31" s="33"/>
     </row>
-    <row r="32" spans="1:13" ht="14.1" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A32" s="70"/>
-      <c r="B32" s="62" t="s">
+    <row r="32" spans="1:13" ht="14.15" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A32" s="73"/>
+      <c r="B32" s="65" t="s">
         <v>53</v>
       </c>
-      <c r="C32" s="63"/>
-      <c r="D32" s="63"/>
-      <c r="E32" s="63"/>
-      <c r="F32" s="63"/>
-      <c r="G32" s="63"/>
-      <c r="H32" s="63"/>
-      <c r="I32" s="63"/>
-      <c r="J32" s="63"/>
+      <c r="C32" s="66"/>
+      <c r="D32" s="66"/>
+      <c r="E32" s="66"/>
+      <c r="F32" s="66"/>
+      <c r="G32" s="66"/>
+      <c r="H32" s="66"/>
+      <c r="I32" s="66"/>
+      <c r="J32" s="66"/>
       <c r="K32" s="27"/>
       <c r="L32" s="28"/>
       <c r="M32" s="33"/>
     </row>
-    <row r="33" spans="1:13" ht="17.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A33" s="70"/>
-      <c r="B33" s="89" t="s">
+    <row r="33" spans="1:13" ht="17.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A33" s="73"/>
+      <c r="B33" s="92" t="s">
         <v>14</v>
       </c>
-      <c r="C33" s="90"/>
-      <c r="D33" s="90"/>
-      <c r="E33" s="90"/>
-      <c r="F33" s="90"/>
-      <c r="G33" s="90"/>
-      <c r="H33" s="90"/>
-      <c r="I33" s="90"/>
-      <c r="J33" s="90"/>
-      <c r="K33" s="91"/>
+      <c r="C33" s="93"/>
+      <c r="D33" s="93"/>
+      <c r="E33" s="93"/>
+      <c r="F33" s="93"/>
+      <c r="G33" s="93"/>
+      <c r="H33" s="93"/>
+      <c r="I33" s="93"/>
+      <c r="J33" s="93"/>
+      <c r="K33" s="94"/>
       <c r="L33" s="14" t="s">
         <v>7</v>
       </c>
@@ -2339,192 +2344,192 @@
         <v>8</v>
       </c>
     </row>
-    <row r="34" spans="1:13" ht="21.95" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A34" s="70"/>
-      <c r="B34" s="64" t="s">
+    <row r="34" spans="1:13" ht="22" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A34" s="73"/>
+      <c r="B34" s="67" t="s">
         <v>54</v>
       </c>
-      <c r="C34" s="65"/>
-      <c r="D34" s="65"/>
-      <c r="E34" s="65"/>
-      <c r="F34" s="65"/>
-      <c r="G34" s="65"/>
-      <c r="H34" s="65"/>
-      <c r="I34" s="65"/>
-      <c r="J34" s="65"/>
+      <c r="C34" s="68"/>
+      <c r="D34" s="68"/>
+      <c r="E34" s="68"/>
+      <c r="F34" s="68"/>
+      <c r="G34" s="68"/>
+      <c r="H34" s="68"/>
+      <c r="I34" s="68"/>
+      <c r="J34" s="68"/>
       <c r="K34" s="26"/>
       <c r="L34" s="28"/>
       <c r="M34" s="33"/>
     </row>
-    <row r="35" spans="1:13" ht="18" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A35" s="70"/>
-      <c r="B35" s="49" t="s">
+    <row r="35" spans="1:13" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A35" s="73"/>
+      <c r="B35" s="52" t="s">
         <v>55</v>
       </c>
-      <c r="C35" s="50"/>
-      <c r="D35" s="50"/>
-      <c r="E35" s="50"/>
-      <c r="F35" s="50"/>
-      <c r="G35" s="50"/>
-      <c r="H35" s="50"/>
-      <c r="I35" s="50"/>
-      <c r="J35" s="50"/>
+      <c r="C35" s="53"/>
+      <c r="D35" s="53"/>
+      <c r="E35" s="53"/>
+      <c r="F35" s="53"/>
+      <c r="G35" s="53"/>
+      <c r="H35" s="53"/>
+      <c r="I35" s="53"/>
+      <c r="J35" s="53"/>
       <c r="K35" s="25"/>
       <c r="L35" s="28"/>
       <c r="M35" s="33"/>
     </row>
-    <row r="36" spans="1:13" ht="18" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A36" s="70"/>
-      <c r="B36" s="49" t="s">
+    <row r="36" spans="1:13" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A36" s="73"/>
+      <c r="B36" s="52" t="s">
         <v>29</v>
       </c>
-      <c r="C36" s="50"/>
-      <c r="D36" s="50"/>
-      <c r="E36" s="50"/>
-      <c r="F36" s="50"/>
-      <c r="G36" s="50"/>
-      <c r="H36" s="50"/>
-      <c r="I36" s="50"/>
-      <c r="J36" s="50"/>
+      <c r="C36" s="53"/>
+      <c r="D36" s="53"/>
+      <c r="E36" s="53"/>
+      <c r="F36" s="53"/>
+      <c r="G36" s="53"/>
+      <c r="H36" s="53"/>
+      <c r="I36" s="53"/>
+      <c r="J36" s="53"/>
       <c r="K36" s="25"/>
       <c r="L36" s="28"/>
       <c r="M36" s="33"/>
     </row>
-    <row r="37" spans="1:13" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A37" s="71"/>
-      <c r="B37" s="62" t="s">
+    <row r="37" spans="1:13" ht="20.149999999999999" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A37" s="74"/>
+      <c r="B37" s="65" t="s">
         <v>11</v>
       </c>
-      <c r="C37" s="63"/>
-      <c r="D37" s="63"/>
-      <c r="E37" s="63"/>
-      <c r="F37" s="63"/>
-      <c r="G37" s="63"/>
-      <c r="H37" s="63"/>
-      <c r="I37" s="63"/>
-      <c r="J37" s="63"/>
+      <c r="C37" s="66"/>
+      <c r="D37" s="66"/>
+      <c r="E37" s="66"/>
+      <c r="F37" s="66"/>
+      <c r="G37" s="66"/>
+      <c r="H37" s="66"/>
+      <c r="I37" s="66"/>
+      <c r="J37" s="66"/>
       <c r="K37" s="37"/>
       <c r="L37" s="34"/>
       <c r="M37" s="35"/>
     </row>
-    <row r="38" spans="1:13" s="46" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="38" spans="1:13" s="46" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A38" s="45" t="s">
         <v>57</v>
       </c>
     </row>
-    <row r="43" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A43" s="66" t="s">
+    <row r="43" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A43" s="69" t="s">
         <v>4</v>
       </c>
-      <c r="B43" s="67"/>
-      <c r="C43" s="67"/>
-      <c r="D43" s="68"/>
+      <c r="B43" s="70"/>
+      <c r="C43" s="70"/>
+      <c r="D43" s="71"/>
       <c r="E43" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="G43" s="66" t="s">
+      <c r="G43" s="69" t="s">
         <v>4</v>
       </c>
-      <c r="H43" s="67"/>
-      <c r="I43" s="67"/>
-      <c r="J43" s="67"/>
-      <c r="K43" s="67"/>
-      <c r="L43" s="68"/>
+      <c r="H43" s="70"/>
+      <c r="I43" s="70"/>
+      <c r="J43" s="70"/>
+      <c r="K43" s="70"/>
+      <c r="L43" s="71"/>
       <c r="M43" s="3" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="44" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="44" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A44" s="48">
         <v>1</v>
       </c>
-      <c r="B44" s="58"/>
-      <c r="C44" s="59"/>
-      <c r="D44" s="60"/>
+      <c r="B44" s="61"/>
+      <c r="C44" s="62"/>
+      <c r="D44" s="63"/>
       <c r="E44" s="4"/>
-      <c r="G44" s="61">
+      <c r="G44" s="64">
         <v>6</v>
       </c>
-      <c r="H44" s="61"/>
-      <c r="I44" s="61"/>
-      <c r="J44" s="61"/>
-      <c r="K44" s="61"/>
-      <c r="L44" s="61"/>
+      <c r="H44" s="64"/>
+      <c r="I44" s="64"/>
+      <c r="J44" s="64"/>
+      <c r="K44" s="64"/>
+      <c r="L44" s="64"/>
       <c r="M44" s="1"/>
     </row>
-    <row r="45" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="45" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A45" s="48">
         <v>2</v>
       </c>
-      <c r="B45" s="58"/>
-      <c r="C45" s="59"/>
-      <c r="D45" s="60"/>
+      <c r="B45" s="61"/>
+      <c r="C45" s="62"/>
+      <c r="D45" s="63"/>
       <c r="E45" s="4"/>
-      <c r="G45" s="61">
+      <c r="G45" s="64">
         <v>7</v>
       </c>
-      <c r="H45" s="61"/>
-      <c r="I45" s="61"/>
-      <c r="J45" s="61"/>
-      <c r="K45" s="61"/>
-      <c r="L45" s="61"/>
+      <c r="H45" s="64"/>
+      <c r="I45" s="64"/>
+      <c r="J45" s="64"/>
+      <c r="K45" s="64"/>
+      <c r="L45" s="64"/>
       <c r="M45" s="1"/>
     </row>
-    <row r="46" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="46" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A46" s="48">
         <v>3</v>
       </c>
-      <c r="B46" s="58"/>
-      <c r="C46" s="59"/>
-      <c r="D46" s="60"/>
+      <c r="B46" s="61"/>
+      <c r="C46" s="62"/>
+      <c r="D46" s="63"/>
       <c r="E46" s="4"/>
-      <c r="G46" s="61">
+      <c r="G46" s="64">
         <v>8</v>
       </c>
-      <c r="H46" s="61"/>
-      <c r="I46" s="61"/>
-      <c r="J46" s="61"/>
-      <c r="K46" s="61"/>
-      <c r="L46" s="61"/>
+      <c r="H46" s="64"/>
+      <c r="I46" s="64"/>
+      <c r="J46" s="64"/>
+      <c r="K46" s="64"/>
+      <c r="L46" s="64"/>
       <c r="M46" s="1"/>
     </row>
-    <row r="47" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="47" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A47" s="48">
         <v>4</v>
       </c>
-      <c r="B47" s="58"/>
-      <c r="C47" s="59"/>
-      <c r="D47" s="60"/>
+      <c r="B47" s="61"/>
+      <c r="C47" s="62"/>
+      <c r="D47" s="63"/>
       <c r="E47" s="4"/>
-      <c r="G47" s="61">
+      <c r="G47" s="64">
         <v>9</v>
       </c>
-      <c r="H47" s="61"/>
-      <c r="I47" s="61"/>
-      <c r="J47" s="61"/>
-      <c r="K47" s="61"/>
-      <c r="L47" s="61"/>
+      <c r="H47" s="64"/>
+      <c r="I47" s="64"/>
+      <c r="J47" s="64"/>
+      <c r="K47" s="64"/>
+      <c r="L47" s="64"/>
       <c r="M47" s="1"/>
     </row>
-    <row r="48" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="48" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A48" s="48">
         <v>5</v>
       </c>
-      <c r="B48" s="58"/>
-      <c r="C48" s="59"/>
-      <c r="D48" s="60"/>
+      <c r="B48" s="61"/>
+      <c r="C48" s="62"/>
+      <c r="D48" s="63"/>
       <c r="E48" s="4"/>
-      <c r="G48" s="61">
+      <c r="G48" s="64">
         <v>10</v>
       </c>
-      <c r="H48" s="61"/>
-      <c r="I48" s="61"/>
-      <c r="J48" s="61"/>
-      <c r="K48" s="61"/>
-      <c r="L48" s="61"/>
+      <c r="H48" s="64"/>
+      <c r="I48" s="64"/>
+      <c r="J48" s="64"/>
+      <c r="K48" s="64"/>
+      <c r="L48" s="64"/>
       <c r="M48" s="1"/>
     </row>
-    <row r="49" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="49" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A49" s="21"/>
       <c r="B49" s="22"/>
       <c r="C49" s="22"/>
@@ -2538,7 +2543,7 @@
       <c r="L49" s="21"/>
       <c r="M49" s="24"/>
     </row>
-    <row r="50" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="50" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A50" s="21"/>
       <c r="B50" s="22"/>
       <c r="C50" s="22"/>
@@ -2552,344 +2557,344 @@
       <c r="L50" s="21"/>
       <c r="M50" s="24"/>
     </row>
-    <row r="51" spans="1:13" ht="15" thickBot="1" x14ac:dyDescent="0.25"/>
-    <row r="52" spans="1:13" ht="15.75" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A52" s="92" t="s">
+    <row r="51" spans="1:13" ht="14.5" thickBot="1" x14ac:dyDescent="0.35"/>
+    <row r="52" spans="1:13" ht="14.5" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A52" s="95" t="s">
         <v>27</v>
       </c>
-      <c r="B52" s="93"/>
-      <c r="C52" s="93"/>
-      <c r="D52" s="93"/>
-      <c r="E52" s="93"/>
-      <c r="F52" s="93"/>
-      <c r="G52" s="93"/>
-      <c r="H52" s="93"/>
-      <c r="I52" s="93"/>
-      <c r="J52" s="93"/>
-      <c r="K52" s="93"/>
-      <c r="L52" s="93"/>
-      <c r="M52" s="94"/>
-    </row>
-    <row r="53" spans="1:13" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B52" s="96"/>
+      <c r="C52" s="96"/>
+      <c r="D52" s="96"/>
+      <c r="E52" s="96"/>
+      <c r="F52" s="96"/>
+      <c r="G52" s="96"/>
+      <c r="H52" s="96"/>
+      <c r="I52" s="96"/>
+      <c r="J52" s="96"/>
+      <c r="K52" s="96"/>
+      <c r="L52" s="96"/>
+      <c r="M52" s="97"/>
+    </row>
+    <row r="53" spans="1:13" ht="14.5" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A53" s="12" t="s">
         <v>10</v>
       </c>
-      <c r="B53" s="53" t="s">
+      <c r="B53" s="56" t="s">
         <v>9</v>
       </c>
-      <c r="C53" s="54"/>
-      <c r="D53" s="54"/>
-      <c r="E53" s="54"/>
-      <c r="F53" s="54"/>
-      <c r="G53" s="54"/>
-      <c r="H53" s="54"/>
-      <c r="I53" s="54"/>
-      <c r="J53" s="54"/>
-      <c r="K53" s="54"/>
-      <c r="L53" s="54"/>
-      <c r="M53" s="55"/>
-    </row>
-    <row r="54" spans="1:13" ht="15" x14ac:dyDescent="0.25">
+      <c r="C53" s="57"/>
+      <c r="D53" s="57"/>
+      <c r="E53" s="57"/>
+      <c r="F53" s="57"/>
+      <c r="G53" s="57"/>
+      <c r="H53" s="57"/>
+      <c r="I53" s="57"/>
+      <c r="J53" s="57"/>
+      <c r="K53" s="57"/>
+      <c r="L53" s="57"/>
+      <c r="M53" s="58"/>
+    </row>
+    <row r="54" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A54" s="7"/>
-      <c r="B54" s="56"/>
-      <c r="C54" s="56"/>
-      <c r="D54" s="56"/>
-      <c r="E54" s="56"/>
-      <c r="F54" s="56"/>
-      <c r="G54" s="56"/>
-      <c r="H54" s="56"/>
-      <c r="I54" s="56"/>
-      <c r="J54" s="56"/>
-      <c r="K54" s="56"/>
-      <c r="L54" s="56"/>
-      <c r="M54" s="56"/>
-    </row>
-    <row r="55" spans="1:13" ht="15" x14ac:dyDescent="0.25">
+      <c r="B54" s="59"/>
+      <c r="C54" s="59"/>
+      <c r="D54" s="59"/>
+      <c r="E54" s="59"/>
+      <c r="F54" s="59"/>
+      <c r="G54" s="59"/>
+      <c r="H54" s="59"/>
+      <c r="I54" s="59"/>
+      <c r="J54" s="59"/>
+      <c r="K54" s="59"/>
+      <c r="L54" s="59"/>
+      <c r="M54" s="59"/>
+    </row>
+    <row r="55" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A55" s="5"/>
-      <c r="B55" s="52"/>
-      <c r="C55" s="52"/>
-      <c r="D55" s="52"/>
-      <c r="E55" s="52"/>
-      <c r="F55" s="52"/>
-      <c r="G55" s="52"/>
-      <c r="H55" s="52"/>
-      <c r="I55" s="52"/>
-      <c r="J55" s="52"/>
-      <c r="K55" s="52"/>
-      <c r="L55" s="52"/>
-      <c r="M55" s="52"/>
-    </row>
-    <row r="56" spans="1:13" ht="15" x14ac:dyDescent="0.25">
+      <c r="B55" s="55"/>
+      <c r="C55" s="55"/>
+      <c r="D55" s="55"/>
+      <c r="E55" s="55"/>
+      <c r="F55" s="55"/>
+      <c r="G55" s="55"/>
+      <c r="H55" s="55"/>
+      <c r="I55" s="55"/>
+      <c r="J55" s="55"/>
+      <c r="K55" s="55"/>
+      <c r="L55" s="55"/>
+      <c r="M55" s="55"/>
+    </row>
+    <row r="56" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A56" s="5"/>
-      <c r="B56" s="52"/>
-      <c r="C56" s="52"/>
-      <c r="D56" s="52"/>
-      <c r="E56" s="52"/>
-      <c r="F56" s="52"/>
-      <c r="G56" s="52"/>
-      <c r="H56" s="52"/>
-      <c r="I56" s="52"/>
-      <c r="J56" s="52"/>
-      <c r="K56" s="52"/>
-      <c r="L56" s="52"/>
-      <c r="M56" s="52"/>
-    </row>
-    <row r="57" spans="1:13" ht="15" x14ac:dyDescent="0.25">
+      <c r="B56" s="55"/>
+      <c r="C56" s="55"/>
+      <c r="D56" s="55"/>
+      <c r="E56" s="55"/>
+      <c r="F56" s="55"/>
+      <c r="G56" s="55"/>
+      <c r="H56" s="55"/>
+      <c r="I56" s="55"/>
+      <c r="J56" s="55"/>
+      <c r="K56" s="55"/>
+      <c r="L56" s="55"/>
+      <c r="M56" s="55"/>
+    </row>
+    <row r="57" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A57" s="5"/>
-      <c r="B57" s="52"/>
-      <c r="C57" s="52"/>
-      <c r="D57" s="52"/>
-      <c r="E57" s="52"/>
-      <c r="F57" s="52"/>
-      <c r="G57" s="52"/>
-      <c r="H57" s="52"/>
-      <c r="I57" s="52"/>
-      <c r="J57" s="52"/>
-      <c r="K57" s="52"/>
-      <c r="L57" s="52"/>
-      <c r="M57" s="52"/>
-    </row>
-    <row r="58" spans="1:13" ht="15" x14ac:dyDescent="0.25">
+      <c r="B57" s="55"/>
+      <c r="C57" s="55"/>
+      <c r="D57" s="55"/>
+      <c r="E57" s="55"/>
+      <c r="F57" s="55"/>
+      <c r="G57" s="55"/>
+      <c r="H57" s="55"/>
+      <c r="I57" s="55"/>
+      <c r="J57" s="55"/>
+      <c r="K57" s="55"/>
+      <c r="L57" s="55"/>
+      <c r="M57" s="55"/>
+    </row>
+    <row r="58" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A58" s="5"/>
-      <c r="B58" s="52"/>
-      <c r="C58" s="52"/>
-      <c r="D58" s="52"/>
-      <c r="E58" s="52"/>
-      <c r="F58" s="52"/>
-      <c r="G58" s="52"/>
-      <c r="H58" s="52"/>
-      <c r="I58" s="52"/>
-      <c r="J58" s="52"/>
-      <c r="K58" s="52"/>
-      <c r="L58" s="52"/>
-      <c r="M58" s="52"/>
-    </row>
-    <row r="59" spans="1:13" ht="15" x14ac:dyDescent="0.25">
+      <c r="B58" s="55"/>
+      <c r="C58" s="55"/>
+      <c r="D58" s="55"/>
+      <c r="E58" s="55"/>
+      <c r="F58" s="55"/>
+      <c r="G58" s="55"/>
+      <c r="H58" s="55"/>
+      <c r="I58" s="55"/>
+      <c r="J58" s="55"/>
+      <c r="K58" s="55"/>
+      <c r="L58" s="55"/>
+      <c r="M58" s="55"/>
+    </row>
+    <row r="59" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A59" s="5"/>
-      <c r="B59" s="52"/>
-      <c r="C59" s="52"/>
-      <c r="D59" s="52"/>
-      <c r="E59" s="52"/>
-      <c r="F59" s="52"/>
-      <c r="G59" s="52"/>
-      <c r="H59" s="52"/>
-      <c r="I59" s="52"/>
-      <c r="J59" s="52"/>
-      <c r="K59" s="52"/>
-      <c r="L59" s="52"/>
-      <c r="M59" s="52"/>
-    </row>
-    <row r="60" spans="1:13" ht="15" x14ac:dyDescent="0.25">
+      <c r="B59" s="55"/>
+      <c r="C59" s="55"/>
+      <c r="D59" s="55"/>
+      <c r="E59" s="55"/>
+      <c r="F59" s="55"/>
+      <c r="G59" s="55"/>
+      <c r="H59" s="55"/>
+      <c r="I59" s="55"/>
+      <c r="J59" s="55"/>
+      <c r="K59" s="55"/>
+      <c r="L59" s="55"/>
+      <c r="M59" s="55"/>
+    </row>
+    <row r="60" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A60" s="5"/>
-      <c r="B60" s="52"/>
-      <c r="C60" s="52"/>
-      <c r="D60" s="52"/>
-      <c r="E60" s="52"/>
-      <c r="F60" s="52"/>
-      <c r="G60" s="52"/>
-      <c r="H60" s="52"/>
-      <c r="I60" s="52"/>
-      <c r="J60" s="52"/>
-      <c r="K60" s="52"/>
-      <c r="L60" s="52"/>
-      <c r="M60" s="52"/>
-    </row>
-    <row r="61" spans="1:13" ht="15" x14ac:dyDescent="0.25">
+      <c r="B60" s="55"/>
+      <c r="C60" s="55"/>
+      <c r="D60" s="55"/>
+      <c r="E60" s="55"/>
+      <c r="F60" s="55"/>
+      <c r="G60" s="55"/>
+      <c r="H60" s="55"/>
+      <c r="I60" s="55"/>
+      <c r="J60" s="55"/>
+      <c r="K60" s="55"/>
+      <c r="L60" s="55"/>
+      <c r="M60" s="55"/>
+    </row>
+    <row r="61" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A61" s="5"/>
-      <c r="B61" s="52"/>
-      <c r="C61" s="52"/>
-      <c r="D61" s="52"/>
-      <c r="E61" s="52"/>
-      <c r="F61" s="52"/>
-      <c r="G61" s="52"/>
-      <c r="H61" s="52"/>
-      <c r="I61" s="52"/>
-      <c r="J61" s="52"/>
-      <c r="K61" s="52"/>
-      <c r="L61" s="52"/>
-      <c r="M61" s="52"/>
-    </row>
-    <row r="62" spans="1:13" ht="15" x14ac:dyDescent="0.25">
+      <c r="B61" s="55"/>
+      <c r="C61" s="55"/>
+      <c r="D61" s="55"/>
+      <c r="E61" s="55"/>
+      <c r="F61" s="55"/>
+      <c r="G61" s="55"/>
+      <c r="H61" s="55"/>
+      <c r="I61" s="55"/>
+      <c r="J61" s="55"/>
+      <c r="K61" s="55"/>
+      <c r="L61" s="55"/>
+      <c r="M61" s="55"/>
+    </row>
+    <row r="62" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A62" s="5"/>
-      <c r="B62" s="52"/>
-      <c r="C62" s="52"/>
-      <c r="D62" s="52"/>
-      <c r="E62" s="52"/>
-      <c r="F62" s="52"/>
-      <c r="G62" s="52"/>
-      <c r="H62" s="52"/>
-      <c r="I62" s="52"/>
-      <c r="J62" s="52"/>
-      <c r="K62" s="52"/>
-      <c r="L62" s="52"/>
-      <c r="M62" s="52"/>
-    </row>
-    <row r="63" spans="1:13" ht="15" x14ac:dyDescent="0.25">
+      <c r="B62" s="55"/>
+      <c r="C62" s="55"/>
+      <c r="D62" s="55"/>
+      <c r="E62" s="55"/>
+      <c r="F62" s="55"/>
+      <c r="G62" s="55"/>
+      <c r="H62" s="55"/>
+      <c r="I62" s="55"/>
+      <c r="J62" s="55"/>
+      <c r="K62" s="55"/>
+      <c r="L62" s="55"/>
+      <c r="M62" s="55"/>
+    </row>
+    <row r="63" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A63" s="5"/>
-      <c r="B63" s="52"/>
-      <c r="C63" s="52"/>
-      <c r="D63" s="52"/>
-      <c r="E63" s="52"/>
-      <c r="F63" s="52"/>
-      <c r="G63" s="52"/>
-      <c r="H63" s="52"/>
-      <c r="I63" s="52"/>
-      <c r="J63" s="52"/>
-      <c r="K63" s="52"/>
-      <c r="L63" s="52"/>
-      <c r="M63" s="52"/>
-    </row>
-    <row r="64" spans="1:13" ht="15" x14ac:dyDescent="0.25">
+      <c r="B63" s="55"/>
+      <c r="C63" s="55"/>
+      <c r="D63" s="55"/>
+      <c r="E63" s="55"/>
+      <c r="F63" s="55"/>
+      <c r="G63" s="55"/>
+      <c r="H63" s="55"/>
+      <c r="I63" s="55"/>
+      <c r="J63" s="55"/>
+      <c r="K63" s="55"/>
+      <c r="L63" s="55"/>
+      <c r="M63" s="55"/>
+    </row>
+    <row r="64" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A64" s="5"/>
-      <c r="B64" s="52"/>
-      <c r="C64" s="52"/>
-      <c r="D64" s="52"/>
-      <c r="E64" s="52"/>
-      <c r="F64" s="52"/>
-      <c r="G64" s="52"/>
-      <c r="H64" s="52"/>
-      <c r="I64" s="52"/>
-      <c r="J64" s="52"/>
-      <c r="K64" s="52"/>
-      <c r="L64" s="52"/>
-      <c r="M64" s="52"/>
-    </row>
-    <row r="65" spans="1:14" ht="15" x14ac:dyDescent="0.25">
+      <c r="B64" s="55"/>
+      <c r="C64" s="55"/>
+      <c r="D64" s="55"/>
+      <c r="E64" s="55"/>
+      <c r="F64" s="55"/>
+      <c r="G64" s="55"/>
+      <c r="H64" s="55"/>
+      <c r="I64" s="55"/>
+      <c r="J64" s="55"/>
+      <c r="K64" s="55"/>
+      <c r="L64" s="55"/>
+      <c r="M64" s="55"/>
+    </row>
+    <row r="65" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A65" s="5"/>
-      <c r="B65" s="52"/>
-      <c r="C65" s="52"/>
-      <c r="D65" s="52"/>
-      <c r="E65" s="52"/>
-      <c r="F65" s="52"/>
-      <c r="G65" s="52"/>
-      <c r="H65" s="52"/>
-      <c r="I65" s="52"/>
-      <c r="J65" s="52"/>
-      <c r="K65" s="52"/>
-      <c r="L65" s="52"/>
-      <c r="M65" s="52"/>
-    </row>
-    <row r="66" spans="1:14" ht="15" x14ac:dyDescent="0.25">
+      <c r="B65" s="55"/>
+      <c r="C65" s="55"/>
+      <c r="D65" s="55"/>
+      <c r="E65" s="55"/>
+      <c r="F65" s="55"/>
+      <c r="G65" s="55"/>
+      <c r="H65" s="55"/>
+      <c r="I65" s="55"/>
+      <c r="J65" s="55"/>
+      <c r="K65" s="55"/>
+      <c r="L65" s="55"/>
+      <c r="M65" s="55"/>
+    </row>
+    <row r="66" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A66" s="5"/>
-      <c r="B66" s="52"/>
-      <c r="C66" s="52"/>
-      <c r="D66" s="52"/>
-      <c r="E66" s="52"/>
-      <c r="F66" s="52"/>
-      <c r="G66" s="52"/>
-      <c r="H66" s="52"/>
-      <c r="I66" s="52"/>
-      <c r="J66" s="52"/>
-      <c r="K66" s="52"/>
-      <c r="L66" s="52"/>
-      <c r="M66" s="52"/>
-    </row>
-    <row r="67" spans="1:14" ht="15" x14ac:dyDescent="0.25">
+      <c r="B66" s="55"/>
+      <c r="C66" s="55"/>
+      <c r="D66" s="55"/>
+      <c r="E66" s="55"/>
+      <c r="F66" s="55"/>
+      <c r="G66" s="55"/>
+      <c r="H66" s="55"/>
+      <c r="I66" s="55"/>
+      <c r="J66" s="55"/>
+      <c r="K66" s="55"/>
+      <c r="L66" s="55"/>
+      <c r="M66" s="55"/>
+    </row>
+    <row r="67" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A67" s="5"/>
-      <c r="B67" s="52"/>
-      <c r="C67" s="52"/>
-      <c r="D67" s="52"/>
-      <c r="E67" s="52"/>
-      <c r="F67" s="52"/>
-      <c r="G67" s="52"/>
-      <c r="H67" s="52"/>
-      <c r="I67" s="52"/>
-      <c r="J67" s="52"/>
-      <c r="K67" s="52"/>
-      <c r="L67" s="52"/>
-      <c r="M67" s="52"/>
-    </row>
-    <row r="68" spans="1:14" ht="15" x14ac:dyDescent="0.25">
+      <c r="B67" s="55"/>
+      <c r="C67" s="55"/>
+      <c r="D67" s="55"/>
+      <c r="E67" s="55"/>
+      <c r="F67" s="55"/>
+      <c r="G67" s="55"/>
+      <c r="H67" s="55"/>
+      <c r="I67" s="55"/>
+      <c r="J67" s="55"/>
+      <c r="K67" s="55"/>
+      <c r="L67" s="55"/>
+      <c r="M67" s="55"/>
+    </row>
+    <row r="68" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A68" s="5"/>
-      <c r="B68" s="52"/>
-      <c r="C68" s="52"/>
-      <c r="D68" s="52"/>
-      <c r="E68" s="52"/>
-      <c r="F68" s="52"/>
-      <c r="G68" s="52"/>
-      <c r="H68" s="52"/>
-      <c r="I68" s="52"/>
-      <c r="J68" s="52"/>
-      <c r="K68" s="52"/>
-      <c r="L68" s="52"/>
-      <c r="M68" s="52"/>
-    </row>
-    <row r="69" spans="1:14" ht="15" x14ac:dyDescent="0.25">
+      <c r="B68" s="55"/>
+      <c r="C68" s="55"/>
+      <c r="D68" s="55"/>
+      <c r="E68" s="55"/>
+      <c r="F68" s="55"/>
+      <c r="G68" s="55"/>
+      <c r="H68" s="55"/>
+      <c r="I68" s="55"/>
+      <c r="J68" s="55"/>
+      <c r="K68" s="55"/>
+      <c r="L68" s="55"/>
+      <c r="M68" s="55"/>
+    </row>
+    <row r="69" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A69" s="5"/>
-      <c r="B69" s="52"/>
-      <c r="C69" s="52"/>
-      <c r="D69" s="52"/>
-      <c r="E69" s="52"/>
-      <c r="F69" s="52"/>
-      <c r="G69" s="52"/>
-      <c r="H69" s="52"/>
-      <c r="I69" s="52"/>
-      <c r="J69" s="52"/>
-      <c r="K69" s="52"/>
-      <c r="L69" s="52"/>
-      <c r="M69" s="52"/>
-    </row>
-    <row r="70" spans="1:14" ht="15" x14ac:dyDescent="0.25">
+      <c r="B69" s="55"/>
+      <c r="C69" s="55"/>
+      <c r="D69" s="55"/>
+      <c r="E69" s="55"/>
+      <c r="F69" s="55"/>
+      <c r="G69" s="55"/>
+      <c r="H69" s="55"/>
+      <c r="I69" s="55"/>
+      <c r="J69" s="55"/>
+      <c r="K69" s="55"/>
+      <c r="L69" s="55"/>
+      <c r="M69" s="55"/>
+    </row>
+    <row r="70" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A70" s="5"/>
-      <c r="B70" s="52"/>
-      <c r="C70" s="52"/>
-      <c r="D70" s="52"/>
-      <c r="E70" s="52"/>
-      <c r="F70" s="52"/>
-      <c r="G70" s="52"/>
-      <c r="H70" s="52"/>
-      <c r="I70" s="52"/>
-      <c r="J70" s="52"/>
-      <c r="K70" s="52"/>
-      <c r="L70" s="52"/>
-      <c r="M70" s="52"/>
-    </row>
-    <row r="71" spans="1:14" ht="15" x14ac:dyDescent="0.25">
+      <c r="B70" s="55"/>
+      <c r="C70" s="55"/>
+      <c r="D70" s="55"/>
+      <c r="E70" s="55"/>
+      <c r="F70" s="55"/>
+      <c r="G70" s="55"/>
+      <c r="H70" s="55"/>
+      <c r="I70" s="55"/>
+      <c r="J70" s="55"/>
+      <c r="K70" s="55"/>
+      <c r="L70" s="55"/>
+      <c r="M70" s="55"/>
+    </row>
+    <row r="71" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A71" s="5"/>
-      <c r="B71" s="52"/>
-      <c r="C71" s="52"/>
-      <c r="D71" s="52"/>
-      <c r="E71" s="52"/>
-      <c r="F71" s="52"/>
-      <c r="G71" s="52"/>
-      <c r="H71" s="52"/>
-      <c r="I71" s="52"/>
-      <c r="J71" s="52"/>
-      <c r="K71" s="52"/>
-      <c r="L71" s="52"/>
-      <c r="M71" s="52"/>
-    </row>
-    <row r="72" spans="1:14" ht="15" x14ac:dyDescent="0.25">
+      <c r="B71" s="55"/>
+      <c r="C71" s="55"/>
+      <c r="D71" s="55"/>
+      <c r="E71" s="55"/>
+      <c r="F71" s="55"/>
+      <c r="G71" s="55"/>
+      <c r="H71" s="55"/>
+      <c r="I71" s="55"/>
+      <c r="J71" s="55"/>
+      <c r="K71" s="55"/>
+      <c r="L71" s="55"/>
+      <c r="M71" s="55"/>
+    </row>
+    <row r="72" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A72" s="5"/>
-      <c r="B72" s="52"/>
-      <c r="C72" s="52"/>
-      <c r="D72" s="52"/>
-      <c r="E72" s="52"/>
-      <c r="F72" s="52"/>
-      <c r="G72" s="52"/>
-      <c r="H72" s="52"/>
-      <c r="I72" s="52"/>
-      <c r="J72" s="52"/>
-      <c r="K72" s="52"/>
-      <c r="L72" s="52"/>
-      <c r="M72" s="52"/>
-    </row>
-    <row r="73" spans="1:14" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B72" s="55"/>
+      <c r="C72" s="55"/>
+      <c r="D72" s="55"/>
+      <c r="E72" s="55"/>
+      <c r="F72" s="55"/>
+      <c r="G72" s="55"/>
+      <c r="H72" s="55"/>
+      <c r="I72" s="55"/>
+      <c r="J72" s="55"/>
+      <c r="K72" s="55"/>
+      <c r="L72" s="55"/>
+      <c r="M72" s="55"/>
+    </row>
+    <row r="73" spans="1:14" ht="14.5" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A73" s="6"/>
-      <c r="B73" s="57"/>
-      <c r="C73" s="57"/>
-      <c r="D73" s="57"/>
-      <c r="E73" s="57"/>
-      <c r="F73" s="57"/>
-      <c r="G73" s="57"/>
-      <c r="H73" s="57"/>
-      <c r="I73" s="57"/>
-      <c r="J73" s="57"/>
-      <c r="K73" s="57"/>
-      <c r="L73" s="57"/>
-      <c r="M73" s="57"/>
-    </row>
-    <row r="74" spans="1:14" ht="15" x14ac:dyDescent="0.25">
+      <c r="B73" s="60"/>
+      <c r="C73" s="60"/>
+      <c r="D73" s="60"/>
+      <c r="E73" s="60"/>
+      <c r="F73" s="60"/>
+      <c r="G73" s="60"/>
+      <c r="H73" s="60"/>
+      <c r="I73" s="60"/>
+      <c r="J73" s="60"/>
+      <c r="K73" s="60"/>
+      <c r="L73" s="60"/>
+      <c r="M73" s="60"/>
+    </row>
+    <row r="74" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A74" s="11"/>
       <c r="B74" s="8"/>
       <c r="C74" s="8"/>
@@ -2904,7 +2909,7 @@
       <c r="L74" s="8"/>
       <c r="M74" s="8"/>
     </row>
-    <row r="75" spans="1:14" ht="15" x14ac:dyDescent="0.25">
+    <row r="75" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A75" s="11"/>
       <c r="B75" s="8"/>
       <c r="C75" s="8"/>
@@ -2919,7 +2924,7 @@
       <c r="L75" s="8"/>
       <c r="M75" s="8"/>
     </row>
-    <row r="76" spans="1:14" ht="15" x14ac:dyDescent="0.25">
+    <row r="76" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A76" s="11"/>
       <c r="B76" s="8"/>
       <c r="C76" s="8"/>
@@ -2934,7 +2939,7 @@
       <c r="L76" s="8"/>
       <c r="M76" s="8"/>
     </row>
-    <row r="77" spans="1:14" ht="15" x14ac:dyDescent="0.25">
+    <row r="77" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A77" s="11"/>
       <c r="B77" s="8"/>
       <c r="C77" s="8"/>
@@ -2949,7 +2954,7 @@
       <c r="L77" s="8"/>
       <c r="M77" s="8"/>
     </row>
-    <row r="78" spans="1:14" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="78" spans="1:14" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A78" s="39"/>
       <c r="B78" s="40"/>
       <c r="C78" s="40"/>
@@ -2961,18 +2966,18 @@
       <c r="L78" s="39"/>
       <c r="M78" s="39"/>
     </row>
-    <row r="79" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A79" s="51" t="s">
+    <row r="79" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A79" s="54" t="s">
         <v>26</v>
       </c>
-      <c r="B79" s="51"/>
-      <c r="C79" s="51"/>
+      <c r="B79" s="54"/>
+      <c r="C79" s="54"/>
       <c r="D79" s="42"/>
-      <c r="E79" s="88" t="s">
+      <c r="E79" s="91" t="s">
         <v>33</v>
       </c>
-      <c r="F79" s="88"/>
-      <c r="G79" s="88"/>
+      <c r="F79" s="91"/>
+      <c r="G79" s="91"/>
       <c r="H79" s="43"/>
       <c r="I79" s="43"/>
       <c r="J79" s="41" t="s">
@@ -2983,16 +2988,16 @@
       <c r="M79" s="44"/>
       <c r="N79" s="38"/>
     </row>
-    <row r="80" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A80" s="51" t="s">
+    <row r="80" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A80" s="54" t="s">
         <v>31</v>
       </c>
-      <c r="B80" s="51"/>
-      <c r="C80" s="51"/>
+      <c r="B80" s="54"/>
+      <c r="C80" s="54"/>
       <c r="D80" s="42"/>
-      <c r="E80" s="88"/>
-      <c r="F80" s="88"/>
-      <c r="G80" s="88"/>
+      <c r="E80" s="91"/>
+      <c r="F80" s="91"/>
+      <c r="G80" s="91"/>
       <c r="H80" s="43"/>
       <c r="I80" s="43"/>
       <c r="J80" s="42"/>
@@ -3000,10 +3005,10 @@
       <c r="L80" s="42"/>
       <c r="M80" s="42"/>
     </row>
-    <row r="81" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A81" s="51"/>
-      <c r="B81" s="51"/>
-      <c r="C81" s="51"/>
+    <row r="81" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A81" s="54"/>
+      <c r="B81" s="54"/>
+      <c r="C81" s="54"/>
       <c r="D81" s="42"/>
       <c r="E81" s="42"/>
       <c r="F81" s="42"/>
@@ -3015,27 +3020,25 @@
       <c r="L81" s="42"/>
       <c r="M81" s="42"/>
     </row>
-    <row r="82" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="82" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A82" s="47"/>
       <c r="B82" s="47"/>
       <c r="C82" s="47"/>
     </row>
-    <row r="83" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="83" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A83" s="45" t="s">
         <v>57</v>
       </c>
       <c r="B83" s="46"/>
     </row>
-    <row r="97" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="97" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A97" s="45"/>
     </row>
   </sheetData>
-  <mergeCells count="87">
-    <mergeCell ref="G44:H44"/>
+  <mergeCells count="88">
     <mergeCell ref="I44:L44"/>
     <mergeCell ref="B31:J31"/>
     <mergeCell ref="A6:M7"/>
-    <mergeCell ref="A1:L1"/>
     <mergeCell ref="M1:M4"/>
     <mergeCell ref="B28:J28"/>
     <mergeCell ref="A2:C2"/>
@@ -3063,7 +3066,6 @@
     <mergeCell ref="A8:M9"/>
     <mergeCell ref="B29:J29"/>
     <mergeCell ref="B30:J30"/>
-    <mergeCell ref="B34:J34"/>
     <mergeCell ref="B35:J35"/>
     <mergeCell ref="G45:H45"/>
     <mergeCell ref="A43:D43"/>
@@ -3079,6 +3081,16 @@
     <mergeCell ref="B14:J14"/>
     <mergeCell ref="B15:J15"/>
     <mergeCell ref="B16:J16"/>
+    <mergeCell ref="G44:H44"/>
+    <mergeCell ref="B26:J26"/>
+    <mergeCell ref="B27:J27"/>
+    <mergeCell ref="B19:J19"/>
+    <mergeCell ref="B21:J21"/>
+    <mergeCell ref="B34:J34"/>
+    <mergeCell ref="B68:M68"/>
+    <mergeCell ref="B69:M69"/>
+    <mergeCell ref="B70:M70"/>
+    <mergeCell ref="B71:M71"/>
     <mergeCell ref="B17:J17"/>
     <mergeCell ref="B18:J18"/>
     <mergeCell ref="B58:M58"/>
@@ -3091,20 +3103,6 @@
     <mergeCell ref="G46:H46"/>
     <mergeCell ref="I46:L46"/>
     <mergeCell ref="B25:J25"/>
-    <mergeCell ref="B26:J26"/>
-    <mergeCell ref="B27:J27"/>
-    <mergeCell ref="B19:J19"/>
-    <mergeCell ref="B21:J21"/>
-    <mergeCell ref="B73:M73"/>
-    <mergeCell ref="B66:M66"/>
-    <mergeCell ref="B67:M67"/>
-    <mergeCell ref="B68:M68"/>
-    <mergeCell ref="B69:M69"/>
-    <mergeCell ref="B70:M70"/>
-    <mergeCell ref="B71:M71"/>
-    <mergeCell ref="B22:J22"/>
-    <mergeCell ref="B23:J23"/>
-    <mergeCell ref="B24:J24"/>
     <mergeCell ref="A79:C79"/>
     <mergeCell ref="B65:M65"/>
     <mergeCell ref="B57:M57"/>
@@ -3118,10 +3116,18 @@
     <mergeCell ref="B63:M63"/>
     <mergeCell ref="B64:M64"/>
     <mergeCell ref="B72:M72"/>
+    <mergeCell ref="B73:M73"/>
+    <mergeCell ref="B66:M66"/>
+    <mergeCell ref="B67:M67"/>
+    <mergeCell ref="A1:I1"/>
+    <mergeCell ref="K1:L1"/>
+    <mergeCell ref="B22:J22"/>
+    <mergeCell ref="B23:J23"/>
+    <mergeCell ref="B24:J24"/>
   </mergeCells>
   <printOptions horizontalCentered="1" verticalCentered="1"/>
   <pageMargins left="0.43307086614173229" right="0.23622047244094491" top="0.19685039370078741" bottom="0.15748031496062992" header="0.31496062992125984" footer="0.31496062992125984"/>
-  <pageSetup scale="86" fitToHeight="0" orientation="landscape" r:id="rId1"/>
+  <pageSetup scale="83" fitToHeight="0" orientation="landscape" r:id="rId1"/>
   <rowBreaks count="2" manualBreakCount="2">
     <brk id="38" max="13" man="1"/>
     <brk id="83" max="13" man="1"/>

</xml_diff>